<commit_message>
added sheet of only data from other worksheets in file to read into R and pivot/clean easier
</commit_message>
<xml_diff>
--- a/data/FY2025 Files/Medicaid/obbb_v6.xlsx
+++ b/data/FY2025 Files/Medicaid/obbb_v6.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pworth\Documents\A_Paulafiles\Research\IGPA\FY2025_report\provider_taxes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleaw\Documents\PhD Fall 2021 - Spring 2022\Merriman RA\Fiscal Futures IGPA\Fiscal-Future-Topics\data\FY2025 Files\Medicaid\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B906211-AC41-4066-BDFC-9B2AFCD353A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A4C46B-28E4-42D3-9EF2-97AC3DA0C138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="912" yWindow="888" windowWidth="19704" windowHeight="10788" activeTab="1" xr2:uid="{83A66CF9-30A3-4BA7-A497-4BAECE955A06}"/>
+    <workbookView xWindow="0" yWindow="3366" windowWidth="17280" windowHeight="8994" xr2:uid="{83A66CF9-30A3-4BA7-A497-4BAECE955A06}"/>
   </bookViews>
   <sheets>
-    <sheet name="Logic_Model" sheetId="1" r:id="rId1"/>
+    <sheet name="data" sheetId="6" r:id="rId1"/>
     <sheet name="Revenue_Forecasts" sheetId="3" r:id="rId2"/>
-    <sheet name="For_Alea" sheetId="4" r:id="rId3"/>
-    <sheet name="Sankey_Alea" sheetId="5" r:id="rId4"/>
+    <sheet name="Logic_Model" sheetId="1" r:id="rId3"/>
+    <sheet name="For_Alea" sheetId="4" r:id="rId4"/>
+    <sheet name="Sankey_Alea" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -98,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="117">
   <si>
     <t>Back of Envelope</t>
   </si>
@@ -443,6 +444,12 @@
   </si>
   <si>
     <t>MCO Assessments</t>
+  </si>
+  <si>
+    <t>est_growth_rate</t>
+  </si>
+  <si>
+    <t>Scenario</t>
   </si>
 </sst>
 </file>
@@ -1409,6 +1416,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1416,7 +1424,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2480,318 +2487,154 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37762FBC-B9CC-4B5A-B87E-7277D49F7C0A}">
-  <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="56.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9753812-F728-4277-BB59-1A228FF63ADE}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="28">
+        <f>2025</f>
+        <v>2025</v>
+      </c>
+      <c r="D1" s="28">
+        <f>C1+1</f>
+        <v>2026</v>
+      </c>
+      <c r="E1" s="28">
+        <f t="shared" ref="E1:K1" si="0">D1+1</f>
+        <v>2027</v>
+      </c>
+      <c r="F1" s="28">
+        <f t="shared" si="0"/>
+        <v>2028</v>
+      </c>
+      <c r="G1" s="28">
+        <f t="shared" si="0"/>
+        <v>2029</v>
+      </c>
+      <c r="H1" s="28">
+        <f t="shared" si="0"/>
+        <v>2030</v>
+      </c>
+      <c r="I1" s="28">
+        <f t="shared" si="0"/>
+        <v>2031</v>
+      </c>
+      <c r="J1" s="28">
+        <f t="shared" si="0"/>
+        <v>2032</v>
+      </c>
+      <c r="K1" s="28">
+        <f t="shared" si="0"/>
+        <v>2033</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="31" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="29">
+        <f>0</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="8"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1">
-        <v>1821.5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="1">
-        <v>2004.6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1">
-        <f>SUM(B6:B7)</f>
-        <v>3826.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="3">
-        <v>4712.6278564699996</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" s="3">
-        <f>For_Alea!$E$10</f>
-        <v>886.54</v>
-      </c>
-      <c r="C10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="1">
-        <f>B8</f>
-        <v>3826.1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="1">
-        <f>B8+B10</f>
-        <v>4712.6399999999994</v>
-      </c>
-      <c r="C13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="1"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="43">
-        <f>B13</f>
-        <v>4712.6399999999994</v>
-      </c>
-      <c r="C15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="9"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" s="1"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="1"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="16">
-        <f>0.05</f>
-        <v>0.05</v>
-      </c>
-      <c r="C21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="1">
-        <f>B15/B21</f>
-        <v>94252.799999999988</v>
-      </c>
-      <c r="C22" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="1"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="9"/>
-      <c r="M24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="10">
-        <v>47027</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" s="12">
-        <v>2029</v>
-      </c>
-      <c r="K26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" s="13">
-        <f>0.75</f>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="16">
-        <f>0.01</f>
-        <v>0.01</v>
-      </c>
-      <c r="C28" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B29" s="14">
-        <f>(1+$B$28)^4*B22</f>
-        <v>98079.841633727992</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B31" s="8"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B32" s="14">
-        <f>B21*B29/4</f>
-        <v>1225.9980204215999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" s="14">
-        <f>B29*(B21-0.005)*3/4</f>
-        <v>3310.1946551383203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B34" s="14">
-        <f>SUM(B32:B33)</f>
-        <v>4536.1926755599197</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B36" s="6"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="14">
-        <f>B21*B29</f>
-        <v>4903.9920816863996</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B38" s="14">
-        <f>B34</f>
-        <v>4536.1926755599197</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B39" s="14">
-        <f>B37-B38</f>
-        <v>367.79940612647988</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>17</v>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30">
+        <v>0</v>
+      </c>
+      <c r="E2" s="30">
+        <v>0</v>
+      </c>
+      <c r="F2" s="30">
+        <v>0</v>
+      </c>
+      <c r="G2" s="30">
+        <v>286.95750000000044</v>
+      </c>
+      <c r="H2" s="30">
+        <v>669.56749999999965</v>
+      </c>
+      <c r="I2" s="30">
+        <v>1052.1774999999993</v>
+      </c>
+      <c r="J2" s="30">
+        <v>1147.8299999999995</v>
+      </c>
+      <c r="K2" s="30">
+        <v>1147.8299999999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="29">
+        <f>0.03</f>
+        <v>0.03</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30">
+        <v>0</v>
+      </c>
+      <c r="E3" s="30">
+        <v>0</v>
+      </c>
+      <c r="F3" s="30">
+        <v>0</v>
+      </c>
+      <c r="G3" s="30">
+        <v>322.97319434557494</v>
+      </c>
+      <c r="H3" s="30">
+        <v>776.21224374386429</v>
+      </c>
+      <c r="I3" s="30">
+        <v>1256.3549602311414</v>
+      </c>
+      <c r="J3" s="30">
+        <v>1411.6861189506285</v>
+      </c>
+      <c r="K3" s="30">
+        <v>1454.0367025191472</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="29">
+        <f>-0.03</f>
+        <v>-0.03</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30">
+        <v>0</v>
+      </c>
+      <c r="E4" s="30">
+        <v>0</v>
+      </c>
+      <c r="F4" s="30">
+        <v>0</v>
+      </c>
+      <c r="G4" s="30">
+        <v>254.04141152557531</v>
+      </c>
+      <c r="H4" s="30">
+        <v>574.98039475288397</v>
+      </c>
+      <c r="I4" s="30">
+        <v>876.43440171618204</v>
+      </c>
+      <c r="J4" s="30">
+        <v>927.42694872512357</v>
+      </c>
+      <c r="K4" s="30">
+        <v>899.60414026337003</v>
       </c>
     </row>
   </sheetData>
@@ -2802,16 +2645,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B115927-DA79-43F3-894D-33B8E43C24B4}">
   <dimension ref="A1:W32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="43.44140625" customWidth="1"/>
-    <col min="3" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="10.88671875" customWidth="1"/>
-    <col min="12" max="12" width="5.44140625" customWidth="1"/>
-    <col min="13" max="13" width="18.21875" customWidth="1"/>
+    <col min="1" max="1" width="43.41796875" customWidth="1"/>
+    <col min="3" max="5" width="9.1015625" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="10.89453125" customWidth="1"/>
+    <col min="12" max="12" width="5.41796875" customWidth="1"/>
+    <col min="13" max="13" width="18.20703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -2820,7 +2663,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
@@ -2829,7 +2672,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
@@ -2837,7 +2680,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -2878,7 +2721,7 @@
         <v>2033</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -2895,7 +2738,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>32</v>
       </c>
@@ -2936,7 +2779,7 @@
         <v>119396.62712701071</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -2974,10 +2817,10 @@
         <v>5969.8313563505362</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
@@ -3018,7 +2861,7 @@
         <v>3.500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="2" t="s">
         <v>39</v>
       </c>
@@ -3059,7 +2902,7 @@
         <v>3.500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>36</v>
       </c>
@@ -3097,7 +2940,7 @@
         <v>4178.8819494453764</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -3108,7 +2951,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
@@ -3146,7 +2989,7 @@
         <v>1790.9494069051598</v>
       </c>
     </row>
-    <row r="15" spans="1:23" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" s="18" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="25" t="s">
         <v>97</v>
       </c>
@@ -3174,7 +3017,7 @@
       <c r="V15" s="26"/>
       <c r="W15" s="26"/>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="27" t="s">
         <v>29</v>
       </c>
@@ -3256,7 +3099,7 @@
         <v>2033</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="27" t="s">
         <v>45</v>
       </c>
@@ -3284,7 +3127,7 @@
       <c r="V17" s="30"/>
       <c r="W17" s="30"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="31" t="s">
         <v>46</v>
       </c>
@@ -3350,7 +3193,7 @@
         <v>1413.791999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="31" t="s">
         <v>47</v>
       </c>
@@ -3416,7 +3259,7 @@
         <v>1790.9494069051598</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="31" t="s">
         <v>48</v>
       </c>
@@ -3482,7 +3325,7 @@
         <v>1108.0500916261381</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="M32" t="s">
         <v>17</v>
       </c>
@@ -3494,20 +3337,340 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37762FBC-B9CC-4B5A-B87E-7277D49F7C0A}">
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="56.7890625" customWidth="1"/>
+    <col min="2" max="2" width="17.3125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="8"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1821.5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2004.6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1">
+        <f>SUM(B6:B7)</f>
+        <v>3826.1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3">
+        <v>4712.6278564699996</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="3">
+        <f>For_Alea!$E$10</f>
+        <v>886.54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="5"/>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="1">
+        <f>B8</f>
+        <v>3826.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" s="1">
+        <f>B8+B10</f>
+        <v>4712.6399999999994</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="5"/>
+      <c r="B14" s="1"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="43">
+        <f>B13</f>
+        <v>4712.6399999999994</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="9"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="16">
+        <f>0.05</f>
+        <v>0.05</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="1">
+        <f>B15/B21</f>
+        <v>94252.799999999988</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="5"/>
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="M24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="10">
+        <v>47027</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="12">
+        <v>2029</v>
+      </c>
+      <c r="K26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="13">
+        <f>0.75</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="16">
+        <f>0.01</f>
+        <v>0.01</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="14">
+        <f>(1+$B$28)^4*B22</f>
+        <v>98079.841633727992</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="8"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" s="14">
+        <f>B21*B29/4</f>
+        <v>1225.9980204215999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="14">
+        <f>B29*(B21-0.005)*3/4</f>
+        <v>3310.1946551383203</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B34" s="14">
+        <f>SUM(B32:B33)</f>
+        <v>4536.1926755599197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" s="6"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37" s="14">
+        <f>B21*B29</f>
+        <v>4903.9920816863996</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" s="14">
+        <f>B34</f>
+        <v>4536.1926755599197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" s="14">
+        <f>B37-B38</f>
+        <v>367.79940612647988</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F61767B-2BB6-41AE-878A-0DB456AEBA59}">
   <dimension ref="A1:K43"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="57.77734375" customWidth="1"/>
+    <col min="1" max="1" width="57.7890625" customWidth="1"/>
     <col min="2" max="4" width="13" style="20" customWidth="1"/>
     <col min="5" max="5" width="15" style="21" customWidth="1"/>
-    <col min="6" max="6" width="66.33203125" customWidth="1"/>
-    <col min="7" max="7" width="3.33203125" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" customWidth="1"/>
-    <col min="11" max="11" width="35.6640625" customWidth="1"/>
+    <col min="6" max="6" width="66.3125" customWidth="1"/>
+    <col min="7" max="7" width="3.3125" customWidth="1"/>
+    <col min="10" max="10" width="16.5234375" customWidth="1"/>
+    <col min="11" max="11" width="35.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
@@ -3515,7 +3678,7 @@
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
@@ -3523,13 +3686,13 @@
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2"/>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="19"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="17" t="s">
         <v>50</v>
       </c>
@@ -3552,7 +3715,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="36" t="s">
         <v>74</v>
       </c>
@@ -3574,7 +3737,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -3603,7 +3766,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -3633,7 +3796,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -3666,7 +3829,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -3698,7 +3861,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -3727,7 +3890,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -3756,7 +3919,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="36" t="s">
         <v>75</v>
       </c>
@@ -3766,7 +3929,7 @@
       <c r="E12" s="34"/>
       <c r="F12" s="35"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="24" t="s">
         <v>76</v>
       </c>
@@ -3780,7 +3943,7 @@
         <v>4712.6278564699996</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="5" t="s">
         <v>70</v>
       </c>
@@ -3797,7 +3960,7 @@
         <v>332.96765653000057</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="11" t="s">
         <v>78</v>
       </c>
@@ -3814,7 +3977,7 @@
         <v>4714.1476030000003</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
         <v>79</v>
       </c>
@@ -3831,7 +3994,7 @@
         <v>4712.6132680000001</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="5" t="s">
         <v>77</v>
       </c>
@@ -3848,7 +4011,7 @@
         <v>-1.4588469999580411E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="38" t="s">
         <v>80</v>
       </c>
@@ -3858,7 +4021,7 @@
       <c r="E18" s="39"/>
       <c r="F18" s="35"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="24" t="s">
         <v>68</v>
       </c>
@@ -3873,7 +4036,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -3881,7 +4044,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -3889,37 +4052,37 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="K24" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>92</v>
       </c>
@@ -3931,22 +4094,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C08B70C-E854-44E1-B702-55CFF500D0D2}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="3" max="3" width="40.21875" customWidth="1"/>
+    <col min="2" max="2" width="32.68359375" customWidth="1"/>
+    <col min="3" max="3" width="40.20703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="C2" s="2" t="s">
         <v>100</v>
       </c>
@@ -3957,7 +4120,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -3974,7 +4137,7 @@
         <v>372.82100400000002</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" s="1"/>
       <c r="C4" t="s">
         <v>104</v>
@@ -3986,7 +4149,7 @@
         <v>1448.6935840000001</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>105</v>
       </c>
@@ -4003,7 +4166,7 @@
         <v>886.54</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>106</v>
       </c>
@@ -4020,7 +4183,7 @@
         <v>23.345963999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="B7" s="1"/>
       <c r="C7" t="s">
         <v>108</v>
@@ -4032,12 +4195,12 @@
         <v>1981.227304</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="B8" s="1"/>
       <c r="D8" s="2"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -4051,10 +4214,10 @@
         <v>4712.6278560000001</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2" t="s">
         <v>113</v>
       </c>
@@ -4065,7 +4228,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>114</v>
       </c>
@@ -4076,7 +4239,7 @@
         <v>372.82100400000002</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>114</v>
       </c>
@@ -4087,7 +4250,7 @@
         <v>1448.6935840000001</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>105</v>
       </c>
@@ -4098,7 +4261,7 @@
         <v>886.54</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2" t="s">
         <v>106</v>
       </c>
@@ -4109,7 +4272,7 @@
         <v>23.345963999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2" t="s">
         <v>106</v>
       </c>
@@ -4120,10 +4283,10 @@
         <v>1981.227304</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" s="1"/>
     </row>
   </sheetData>

</xml_diff>